<commit_message>
Final run completed by satyam
</commit_message>
<xml_diff>
--- a/test-output/HotelList.xlsx
+++ b/test-output/HotelList.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
   <si>
     <t>S.No</t>
   </si>
@@ -78,6 +78,33 @@
   </si>
   <si>
     <t>₹ 149,455</t>
+  </si>
+  <si>
+    <t>Cozy Studio Apartment Spa and Safaris</t>
+  </si>
+  <si>
+    <t>₹ 8733.8</t>
+  </si>
+  <si>
+    <t>₹ 43,669</t>
+  </si>
+  <si>
+    <t>Urbanwoods Hotel Suites by ICON</t>
+  </si>
+  <si>
+    <t>₹ 27292.8</t>
+  </si>
+  <si>
+    <t>₹ 136,464</t>
+  </si>
+  <si>
+    <t>Marina Bay One &amp; Two bedroom, Swimming Pool, gym, workspace ESKAY HOMES Westland's Nairobi</t>
+  </si>
+  <si>
+    <t>₹ 11430.8</t>
+  </si>
+  <si>
+    <t>₹ 57,154</t>
   </si>
 </sst>
 </file>
@@ -122,7 +149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -144,13 +171,13 @@
         <v>4</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -158,13 +185,13 @@
         <v>8</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -172,27 +199,13 @@
         <v>12</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>17</v>
-      </c>
-      <c r="C5" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s" s="0">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes in tc_016 and tc_019
</commit_message>
<xml_diff>
--- a/test-output/HotelList.xlsx
+++ b/test-output/HotelList.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="112">
   <si>
     <t>S.No</t>
   </si>
@@ -183,6 +183,171 @@
   </si>
   <si>
     <t>₹ 150,657</t>
+  </si>
+  <si>
+    <t>₹ 6594.6</t>
+  </si>
+  <si>
+    <t>₹ 32,973</t>
+  </si>
+  <si>
+    <t>Ruaka View Apartments- cozy 2 bedroom</t>
+  </si>
+  <si>
+    <t>₹ 3938.4</t>
+  </si>
+  <si>
+    <t>₹ 19,692</t>
+  </si>
+  <si>
+    <t>kingdom corner suites</t>
+  </si>
+  <si>
+    <t>₹ 8243.2</t>
+  </si>
+  <si>
+    <t>₹ 41,216</t>
+  </si>
+  <si>
+    <t>The Suites Fourways</t>
+  </si>
+  <si>
+    <t>₹ 5358.0</t>
+  </si>
+  <si>
+    <t>₹ 26,790</t>
+  </si>
+  <si>
+    <t>The Curve by the Park Nairobi by TSG</t>
+  </si>
+  <si>
+    <t>₹ 9570.4</t>
+  </si>
+  <si>
+    <t>₹ 47,852</t>
+  </si>
+  <si>
+    <t>Wellivia Suites Serviced Apartments</t>
+  </si>
+  <si>
+    <t>₹ 9159.2</t>
+  </si>
+  <si>
+    <t>₹ 45,796</t>
+  </si>
+  <si>
+    <t>Indesign suits-JkIA</t>
+  </si>
+  <si>
+    <t>₹ 4304.8</t>
+  </si>
+  <si>
+    <t>₹ 21,524</t>
+  </si>
+  <si>
+    <t>Lovely 2-bedroom Serviced Hotel Suites with Pool and Wi-Fi at Skynest</t>
+  </si>
+  <si>
+    <t>₹ 13738.6</t>
+  </si>
+  <si>
+    <t>₹ 68,693</t>
+  </si>
+  <si>
+    <t>Classic residence</t>
+  </si>
+  <si>
+    <t>₹ 9809.4</t>
+  </si>
+  <si>
+    <t>₹ 49,047</t>
+  </si>
+  <si>
+    <t>Trademark Suites at Enaki Town</t>
+  </si>
+  <si>
+    <t>₹ 35571.2</t>
+  </si>
+  <si>
+    <t>₹ 177,856</t>
+  </si>
+  <si>
+    <t>₹ 9392.2</t>
+  </si>
+  <si>
+    <t>₹ 46,961</t>
+  </si>
+  <si>
+    <t>Urban Homes-Two Bedroom Near JKIA Airport</t>
+  </si>
+  <si>
+    <t>₹ 5817.0</t>
+  </si>
+  <si>
+    <t>₹ 29,085</t>
+  </si>
+  <si>
+    <t>₹ 12132.8</t>
+  </si>
+  <si>
+    <t>₹ 60,664</t>
+  </si>
+  <si>
+    <t>₹ 10585.6</t>
+  </si>
+  <si>
+    <t>₹ 52,928</t>
+  </si>
+  <si>
+    <t>₹ 18226.2</t>
+  </si>
+  <si>
+    <t>₹ 91,131</t>
+  </si>
+  <si>
+    <t>₹ 30610.8</t>
+  </si>
+  <si>
+    <t>₹ 153,054</t>
+  </si>
+  <si>
+    <t>₹ 72110.0</t>
+  </si>
+  <si>
+    <t>₹ 360,550</t>
+  </si>
+  <si>
+    <t>Fahari Palace Serviced Apartments</t>
+  </si>
+  <si>
+    <t>₹ 13796.6</t>
+  </si>
+  <si>
+    <t>₹ 68,983</t>
+  </si>
+  <si>
+    <t>Hyatt Place Nairobi Westlands</t>
+  </si>
+  <si>
+    <t>₹ 38743.0</t>
+  </si>
+  <si>
+    <t>₹ 193,715</t>
+  </si>
+  <si>
+    <t>₹ 9732.6</t>
+  </si>
+  <si>
+    <t>₹ 48,663</t>
+  </si>
+  <si>
+    <t>Pridehomes</t>
+  </si>
+  <si>
+    <t>₹ 5605.4</t>
+  </si>
+  <si>
+    <t>₹ 28,027</t>
   </si>
 </sst>
 </file>
@@ -252,10 +417,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>6</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>7</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3">
@@ -263,13 +428,13 @@
         <v>8</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>11</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -277,13 +442,13 @@
         <v>12</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>13</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>14</v>
+        <v>63</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>15</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -291,13 +456,13 @@
         <v>16</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>33</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6">
@@ -305,13 +470,13 @@
         <v>34</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>35</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>36</v>
+        <v>107</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>37</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7">
@@ -319,13 +484,13 @@
         <v>38</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>40</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>41</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -333,13 +498,13 @@
         <v>42</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>43</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>44</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>45</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9">
@@ -347,13 +512,13 @@
         <v>46</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>17</v>
+        <v>74</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>48</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10">
@@ -361,13 +526,13 @@
         <v>49</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>50</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>52</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11">
@@ -375,13 +540,13 @@
         <v>53</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>